<commit_message>
EPBDS-16832 Remove deprecated RulesUtils functions and the locale-dependent format(double)
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/Date.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/Date.xlsx
@@ -461,7 +461,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="397">
   <si>
     <t>_res_</t>
   </si>
@@ -1649,6 +1649,9 @@
   </si>
   <si>
     <t>DATEDIF(1/2/1900  6:00:00 AM,1/1/1900,"YD")</t>
+  </si>
+  <si>
+    <t>return toString(date, "M/d/yy");</t>
   </si>
 </sst>
 </file>
@@ -12275,7 +12278,7 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="79" t="s">
-        <v>12</v>
+        <v>396</v>
       </c>
       <c r="C3" s="79"/>
       <c r="D3" s="79"/>

</xml_diff>